<commit_message>
Show maximum speeds consistently and move measurement conditions to details
</commit_message>
<xml_diff>
--- a/downloads/PM9E1_PM9A1_512GB.xlsx
+++ b/downloads/PM9E1_PM9A1_512GB.xlsx
@@ -777,7 +777,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6,900 / 6,300 MB/s (QD32)</t>
+          <t xml:space="preserve">6,900 MB/s</t>
         </is>
       </c>
       <c r="E9" s="2"/>
@@ -794,7 +794,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5,000 / 1,050 MB/s (QD32)</t>
+          <t xml:space="preserve">5,000 MB/s</t>
         </is>
       </c>
       <c r="E10" s="2"/>
@@ -811,7 +811,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">800K / 500K IOPS (QD32)</t>
+          <t xml:space="preserve">800K IOPS</t>
         </is>
       </c>
       <c r="E11" s="2"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">800K / 250K IOPS (QD32)</t>
+          <t xml:space="preserve">800K IOPS</t>
         </is>
       </c>
       <c r="E12" s="1"/>

</xml_diff>